<commit_message>
BPMCCS with RUPTL data
</commit_message>
<xml_diff>
--- a/InputData/elec/BPMCCS/BAU Pol Mandated Cap Const Sched.xlsx
+++ b/InputData/elec/BPMCCS/BAU Pol Mandated Cap Const Sched.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/elec/BPMCCS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4EBB44A-9B6F-2743-9BDF-77757C7A5BBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9A8CB58-398E-F346-9596-AAF273111E23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -954,8 +954,15 @@
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -963,13 +970,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1257,13 +1257,13 @@
       <c r="A3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="52" t="s">
+      <c r="B3" s="47" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="43"/>
-      <c r="B4" s="53">
+      <c r="B4" s="48">
         <v>2021</v>
       </c>
     </row>
@@ -1290,15 +1290,15 @@
       <c r="B9" s="39"/>
     </row>
     <row r="10" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="47"/>
+      <c r="A10" s="49"/>
       <c r="B10" s="44"/>
     </row>
     <row r="11" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="47"/>
+      <c r="A11" s="49"/>
       <c r="B11" s="44"/>
     </row>
     <row r="12" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A12" s="47"/>
+      <c r="A12" s="49"/>
       <c r="B12" s="44"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -2309,20 +2309,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="50" t="s">
         <v>182</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="41" t="s">
@@ -9341,40 +9341,40 @@
       </c>
     </row>
     <row r="87" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B87" s="48" t="s">
+      <c r="B87" s="51" t="s">
         <v>109</v>
       </c>
-      <c r="C87" s="49"/>
-      <c r="D87" s="49"/>
-      <c r="E87" s="49"/>
-      <c r="F87" s="49"/>
-      <c r="G87" s="49"/>
-      <c r="H87" s="49"/>
-      <c r="I87" s="49"/>
-      <c r="J87" s="49"/>
-      <c r="K87" s="49"/>
-      <c r="L87" s="49"/>
-      <c r="M87" s="49"/>
-      <c r="N87" s="49"/>
-      <c r="O87" s="49"/>
-      <c r="P87" s="49"/>
-      <c r="Q87" s="49"/>
-      <c r="R87" s="49"/>
-      <c r="S87" s="49"/>
-      <c r="T87" s="49"/>
-      <c r="U87" s="49"/>
-      <c r="V87" s="49"/>
-      <c r="W87" s="49"/>
-      <c r="X87" s="49"/>
-      <c r="Y87" s="49"/>
-      <c r="Z87" s="49"/>
-      <c r="AA87" s="49"/>
-      <c r="AB87" s="49"/>
-      <c r="AC87" s="49"/>
-      <c r="AD87" s="49"/>
-      <c r="AE87" s="49"/>
-      <c r="AF87" s="49"/>
-      <c r="AG87" s="49"/>
+      <c r="C87" s="52"/>
+      <c r="D87" s="52"/>
+      <c r="E87" s="52"/>
+      <c r="F87" s="52"/>
+      <c r="G87" s="52"/>
+      <c r="H87" s="52"/>
+      <c r="I87" s="52"/>
+      <c r="J87" s="52"/>
+      <c r="K87" s="52"/>
+      <c r="L87" s="52"/>
+      <c r="M87" s="52"/>
+      <c r="N87" s="52"/>
+      <c r="O87" s="52"/>
+      <c r="P87" s="52"/>
+      <c r="Q87" s="52"/>
+      <c r="R87" s="52"/>
+      <c r="S87" s="52"/>
+      <c r="T87" s="52"/>
+      <c r="U87" s="52"/>
+      <c r="V87" s="52"/>
+      <c r="W87" s="52"/>
+      <c r="X87" s="52"/>
+      <c r="Y87" s="52"/>
+      <c r="Z87" s="52"/>
+      <c r="AA87" s="52"/>
+      <c r="AB87" s="52"/>
+      <c r="AC87" s="52"/>
+      <c r="AD87" s="52"/>
+      <c r="AE87" s="52"/>
+      <c r="AF87" s="52"/>
+      <c r="AG87" s="52"/>
       <c r="AH87" s="21"/>
     </row>
     <row r="88" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -9498,39 +9498,39 @@
       </c>
     </row>
     <row r="112" spans="2:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B112" s="50"/>
-      <c r="C112" s="51"/>
-      <c r="D112" s="51"/>
-      <c r="E112" s="51"/>
-      <c r="F112" s="51"/>
-      <c r="G112" s="51"/>
-      <c r="H112" s="51"/>
-      <c r="I112" s="51"/>
-      <c r="J112" s="51"/>
-      <c r="K112" s="51"/>
-      <c r="L112" s="51"/>
-      <c r="M112" s="51"/>
-      <c r="N112" s="51"/>
-      <c r="O112" s="51"/>
-      <c r="P112" s="51"/>
-      <c r="Q112" s="51"/>
-      <c r="R112" s="51"/>
-      <c r="S112" s="51"/>
-      <c r="T112" s="51"/>
-      <c r="U112" s="51"/>
-      <c r="V112" s="51"/>
-      <c r="W112" s="51"/>
-      <c r="X112" s="51"/>
-      <c r="Y112" s="51"/>
-      <c r="Z112" s="51"/>
-      <c r="AA112" s="51"/>
-      <c r="AB112" s="51"/>
-      <c r="AC112" s="51"/>
-      <c r="AD112" s="51"/>
-      <c r="AE112" s="51"/>
-      <c r="AF112" s="51"/>
-      <c r="AG112" s="51"/>
-      <c r="AH112" s="51"/>
+      <c r="B112" s="53"/>
+      <c r="C112" s="54"/>
+      <c r="D112" s="54"/>
+      <c r="E112" s="54"/>
+      <c r="F112" s="54"/>
+      <c r="G112" s="54"/>
+      <c r="H112" s="54"/>
+      <c r="I112" s="54"/>
+      <c r="J112" s="54"/>
+      <c r="K112" s="54"/>
+      <c r="L112" s="54"/>
+      <c r="M112" s="54"/>
+      <c r="N112" s="54"/>
+      <c r="O112" s="54"/>
+      <c r="P112" s="54"/>
+      <c r="Q112" s="54"/>
+      <c r="R112" s="54"/>
+      <c r="S112" s="54"/>
+      <c r="T112" s="54"/>
+      <c r="U112" s="54"/>
+      <c r="V112" s="54"/>
+      <c r="W112" s="54"/>
+      <c r="X112" s="54"/>
+      <c r="Y112" s="54"/>
+      <c r="Z112" s="54"/>
+      <c r="AA112" s="54"/>
+      <c r="AB112" s="54"/>
+      <c r="AC112" s="54"/>
+      <c r="AD112" s="54"/>
+      <c r="AE112" s="54"/>
+      <c r="AF112" s="54"/>
+      <c r="AG112" s="54"/>
+      <c r="AH112" s="54"/>
     </row>
     <row r="113" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="114" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -9728,39 +9728,39 @@
     <row r="306" spans="2:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="307" spans="2:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="308" spans="2:34" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B308" s="50"/>
-      <c r="C308" s="51"/>
-      <c r="D308" s="51"/>
-      <c r="E308" s="51"/>
-      <c r="F308" s="51"/>
-      <c r="G308" s="51"/>
-      <c r="H308" s="51"/>
-      <c r="I308" s="51"/>
-      <c r="J308" s="51"/>
-      <c r="K308" s="51"/>
-      <c r="L308" s="51"/>
-      <c r="M308" s="51"/>
-      <c r="N308" s="51"/>
-      <c r="O308" s="51"/>
-      <c r="P308" s="51"/>
-      <c r="Q308" s="51"/>
-      <c r="R308" s="51"/>
-      <c r="S308" s="51"/>
-      <c r="T308" s="51"/>
-      <c r="U308" s="51"/>
-      <c r="V308" s="51"/>
-      <c r="W308" s="51"/>
-      <c r="X308" s="51"/>
-      <c r="Y308" s="51"/>
-      <c r="Z308" s="51"/>
-      <c r="AA308" s="51"/>
-      <c r="AB308" s="51"/>
-      <c r="AC308" s="51"/>
-      <c r="AD308" s="51"/>
-      <c r="AE308" s="51"/>
-      <c r="AF308" s="51"/>
-      <c r="AG308" s="51"/>
-      <c r="AH308" s="51"/>
+      <c r="B308" s="53"/>
+      <c r="C308" s="54"/>
+      <c r="D308" s="54"/>
+      <c r="E308" s="54"/>
+      <c r="F308" s="54"/>
+      <c r="G308" s="54"/>
+      <c r="H308" s="54"/>
+      <c r="I308" s="54"/>
+      <c r="J308" s="54"/>
+      <c r="K308" s="54"/>
+      <c r="L308" s="54"/>
+      <c r="M308" s="54"/>
+      <c r="N308" s="54"/>
+      <c r="O308" s="54"/>
+      <c r="P308" s="54"/>
+      <c r="Q308" s="54"/>
+      <c r="R308" s="54"/>
+      <c r="S308" s="54"/>
+      <c r="T308" s="54"/>
+      <c r="U308" s="54"/>
+      <c r="V308" s="54"/>
+      <c r="W308" s="54"/>
+      <c r="X308" s="54"/>
+      <c r="Y308" s="54"/>
+      <c r="Z308" s="54"/>
+      <c r="AA308" s="54"/>
+      <c r="AB308" s="54"/>
+      <c r="AC308" s="54"/>
+      <c r="AD308" s="54"/>
+      <c r="AE308" s="54"/>
+      <c r="AF308" s="54"/>
+      <c r="AG308" s="54"/>
+      <c r="AH308" s="54"/>
     </row>
     <row r="309" spans="2:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="310" spans="2:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>